<commit_message>
Pasos previos por receta + materiales (papel vegetal, carbon, etc.)
Columna PasosPrevios en Comidas (adobo cazon, garbanzos remojo, berenjena
con sal para el amargor + papel vegetal, brasas, descongelar carne...).
Basicos: papel vegetal, papel aluminio, carbon, pastillas, bolsas congelacion.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CompraSanJose.xlsx
+++ b/data/CompraSanJose.xlsx
@@ -3248,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3269,15 +3269,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>PasosPrevios</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Preparacion</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -3300,6 +3305,11 @@
         </is>
       </c>
       <c r="D2" t="inlineStr">
+        <is>
+          <t>Descongela la aguja de vaca la noche antes en la nevera.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>1. Pica pimiento verde, ajos y tomate. En la paellera, sofrie pimiento y ajos; anade la aguja de vaca troceada y el chorizo salpimentados y dora.
 2. Incorpora el tomate natural y rehoga.
@@ -3309,12 +3319,12 @@
 6. Apaga, tapa con un pano y reposa 7-8 min.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-arroces/receta-arroz-campero-tipico-andalucia</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3333,6 +3343,11 @@
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>Con antelacion: lava las laminas de berenjena con agua y sal y dejalas 30-45 min para quitar el amargor; escurre y seca. Hornea o frie las laminas de patata y de berenjena antes de montar. Necesitas papel vegetal de horno.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>1. Lamina las berenjenas, salalas y dejalas sudar; frielas ligeramente y reserva.
 2. Corta las patatas en rodajas y frielas ligeramente para la base.
@@ -3343,12 +3358,12 @@
 7. Hornea 20 min a 160C y gratina 3 min a 220C.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-carnes-y-aves/moussaka-receta-griega</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Con ternera (no cordero); tomate tamizado.</t>
         </is>
@@ -3371,6 +3386,11 @@
         </is>
       </c>
       <c r="D4" t="inlineStr">
+        <is>
+          <t>La noche anterior: deja los garbanzos en remojo (o usa garbanzos ya cocidos). Puedes guisar la carrillera la vispera; gana de un dia para otro.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>1. Trocea la carrillera de ternera, salpimienta y dorala a fuego alto en la cazuela.
 2. Baja el fuego, anade cebolla y pocha 10 min.
@@ -3381,12 +3401,12 @@
 7. Sirve la semola de base y reparte el guiso por encima.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://www.todosacomer.net/recetas/guisos-pasta-arroces/cuscus-con-verduras-y-pollo</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Zanahoria opcional; tomate tamizado (poco).</t>
         </is>
@@ -3408,7 +3428,8 @@
           <t>Paco</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>1. Corta las patatas en rodajas de 1/2 cm; pica ajo y corta cebolla y pimiento verde.
 2. En abundante aceite, frie ajo y luego patatas, cebolla y pimiento; 5 min a fuego fuerte.
@@ -3418,12 +3439,12 @@
 6. Emplata: base de patatas, encima embutidos, huevos fritos y unas lonchas de jamon.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://bonviveur.com/es/recetas/plato-alpujarreno</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Patatas a lo pobre + embutido + huevos.</t>
         </is>
@@ -3446,6 +3467,11 @@
         </is>
       </c>
       <c r="D6" t="inlineStr">
+        <is>
+          <t>Preparalo con antelacion y enfrialo en nevera al menos 2 h antes de servir.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>1. Tritura los tomates (1 kg por cada 6 raciones); no hace falta pelar ni despepitar.
 2. Anade el pan (unos 200 g de telera por cada 6) y deja que se empape 10 min.
@@ -3455,12 +3481,12 @@
 6. De acompanamiento, salpimienta los filetes y hazlos a la plancha 2-3 min por cara.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-sopas-y-cremas/receta-de-salmorejo-cordobes-tradicional</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Acompanamiento elegible; por defecto filetes de ternera.</t>
         </is>
@@ -3482,7 +3508,8 @@
           <t>Manolo</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
         <is>
           <t>1. Corta pan candeal asentado en cubos de 1 cm; humedecelo con agua salada, tapa con un pano y reposa (mejor de un dia para otro).
 2. Frie el chorizo en rodajas y la panceta en dados hasta que suelten grasa; reserva.
@@ -3492,12 +3519,12 @@
 6. Para grupo grande, trabaja por tandas o en perol amplio; sirve muy caliente.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-tradicionales/mejor-receta-migas-pan-chorizo-clasico-potente-como-tradicional</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3516,6 +3543,11 @@
         </is>
       </c>
       <c r="D8" t="inlineStr">
+        <is>
+          <t>Se puede cocinar la vispera; gana de un dia para otro.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>1. Pocha la cebolla en aceite hasta transparente.
 2. Anade ajo, pimenton picante y comino; rehoga.
@@ -3525,12 +3557,12 @@
 6. Rectifica de sal y picante; sirve con arroz blanco y nachos.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-carnes-y-aves/chili-receta-mexicana-con-y-sin-thermomix</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Con guarnicion de arroz.</t>
         </is>
@@ -3553,6 +3585,11 @@
         </is>
       </c>
       <c r="D9" t="inlineStr">
+        <is>
+          <t>Precalienta el horno a 180C. Cubre la bandeja con papel vegetal o engrasala bien.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>1. Precalienta el horno a 180C. Mezcla sal, pimienta y tomillo/romero.
 2. Parte las patatas, hazles cortes y colocalas en la bandeja engrasada.
@@ -3562,12 +3599,12 @@
 6. Trincha, riega con la salsa y sirve; para mas comensales reparte en varias bandejas sin amontonar.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://www.hogarmania.com/cocina/recetas/carnes/pollo-asado-patatas-ensalada-verde-16651.html</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>El 'asado de carne/pescado'.</t>
         </is>
@@ -3589,7 +3626,8 @@
           <t>Paco</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
         <is>
           <t>1. Pica en cuadraditos la cebolla y el pimiento verde; pica una pizca de ajo.
 2. Pocha cebolla, pimiento y ajo en aceite 10-15 min a fuego medio.
@@ -3599,12 +3637,12 @@
 6. Sirve el pisto con los huevos fritos por encima.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-legumbres-y-verduras/pisto-de-pimientos-y-tomates-la-receta-de-mi-abuela</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>RESPALDO: solo cebolla, tomate frito y pimiento verde + huevos.</t>
         </is>
@@ -3627,6 +3665,11 @@
         </is>
       </c>
       <c r="D11" t="inlineStr">
+        <is>
+          <t>Enciende las brasas 30-40 min antes (carbon + pastillas). Ten la carne fresca (sin congelar) y las salsas listas.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>1. Enciende la barbacoa 30-40 min antes; espera a que las brasas esten blanquecinas, sin llama.
 2. Reparte el carbon para calor uniforme; parrilla no muy pegada a las brasas.
@@ -3637,12 +3680,12 @@
 7. NO sales antes: echa la sal SOLO AL FINAL, en el plato.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/cultura-gastronomica/los-9-trucos-imprescindibles-para-convertirte-en-el-maestro-de-las-barbacoas</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Cerdo y embutido. Tope de carne por comensal (RF-26).</t>
         </is>
@@ -3665,6 +3708,11 @@
         </is>
       </c>
       <c r="D12" t="inlineStr">
+        <is>
+          <t>Enciende las brasas 30-40 min antes. Saca el vacuno de la nevera para atemperar. Ten el chimichurri preparado.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>1. Enciende las brasas 30-40 min antes; saca el vacuno de la nevera para atemperar.
 2. Sella el entrecot y el chuleton sobre brasa fuerte ~5 min por cara; una sola vuelta.
@@ -3675,12 +3723,12 @@
 7. Echa la sal AL FINAL para no resecar la carne.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetario/83-mejores-recetas-barbacoa-para-sacar-todo-partido-a-parrilla-este-verano</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Vacuno, pollo y verdura. Tope de carne por comensal (RF-26).</t>
         </is>
@@ -3702,7 +3750,8 @@
           <t>Manolo</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
         <is>
           <t>1. Corta el pollo en tiras y la cebolla y los pimientos en tiras anchas.
 2. Salpimienta el pollo y saltealo en aceite muy caliente; reserva.
@@ -3712,12 +3761,12 @@
 6. Rellena y enrolla; sirve con guacamole, nata agria, queso, tomate y lechuga.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://www.divinacocina.es/fajitas-de-pollo-faciles/</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3731,7 +3780,8 @@
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
         <is>
           <t>1. Usa carne picada fresca; salpimienta.
 2. Mezcla sin amasar en exceso y forma discos regulares.
@@ -3742,12 +3792,12 @@
 7. Monta: pan, lechuga y tomate, hamburguesa, bacon, cebolla y pepinillos, salsa y cierra. Acompana con patatas.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-carnes-y-aves/como-hacer-hamburguesas-caseras</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3761,7 +3811,8 @@
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
         <is>
           <t>1. Mezcla la masa (harina, agua, levadura, sal, aceite) hasta homogenea; reposa 1-3 h.
 2. Divide, bolea y deja reposar; sacala 1-2 h antes si estaba en frio.
@@ -3772,12 +3823,12 @@
 7. Reposa unos minutos; anade oregano y aceite al salir.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-panes/pizza-casera-la-guia-definitiva</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3796,6 +3847,11 @@
         </is>
       </c>
       <c r="D16" t="inlineStr">
+        <is>
+          <t>El dia anterior: adoba el cazon y la rosada (ajo, comino, oregano, pimenton, vinagre de Jerez, laurel y sal) y macera en nevera 8-12 h. Saca a temperatura antes de enharinar.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>1. Adobo del cazon: maja ajo, comino, oregano y pimenton, anade vinagre, laurel y sal.
 2. Corta el cazon en tacos, cubrelo con el adobo y macera en nevera 8 h (mejor toda la noche).
@@ -3806,12 +3862,12 @@
 7. Escurre en papel y sirve al momento con limon.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>https://www.directoalpaladar.com/recetas-de-aperitivos/como-se-hace-el-cazon-en-adobo-receta-de-bienmesabe</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Surtido elegible; incluye adobo y tempura.</t>
         </is>
@@ -3833,7 +3889,8 @@
           <t>Paco</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
         <is>
           <t>1. Sofrie cebolla, pimiento y ajo en aceite; anade tomate natural.
 2. Rehoga el arroz con pimenton y azafran.
@@ -3842,8 +3899,8 @@
 5. Cuece 18 min sin remover; reposa 5 min. Sirve con limon.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>Opcion alternativa de arroz.</t>
         </is>
@@ -11869,7 +11926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12461,6 +12518,116 @@
         </is>
       </c>
       <c r="D27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Papel vegetal de horno</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Rollo</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Papel de aluminio</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Rollo</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Carbon para barbacoa</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Saco</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Pastillas de encendido</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Bolsas de congelacion</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>